<commit_message>
Use SUMIF function to add balues when a certain condition is true: total sales in a region
</commit_message>
<xml_diff>
--- a/Sales_Performance_Analysis.xlsx
+++ b/Sales_Performance_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI-Projects\sales-performance-analysis-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D600EC3A-E168-4CDB-B6CB-2D9151059E19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD19108-D6E8-4AF6-A488-C6CFA3FF5340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="4" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="2" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="133">
   <si>
     <t>Region</t>
   </si>
@@ -434,6 +434,9 @@
   </si>
   <si>
     <t>Lowest Sale</t>
+  </si>
+  <si>
+    <t>Sales</t>
   </si>
 </sst>
 </file>
@@ -1264,22 +1267,28 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D65C6-FEF1-4656-8613-EFBCAEDD2EBF}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
     <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>125</v>
       </c>
       <c r="B1" s="11" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1287,8 +1296,15 @@
         <f>SUM(SalesTable[Total Sales])</f>
         <v>45285</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <f>SUMIF(SalesTable[Region],D2,SalesTable[Total Sales])</f>
+        <v>12045</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>127</v>
       </c>
@@ -1296,8 +1312,15 @@
         <f>SUM(SalesTable[Quantity])</f>
         <v>277</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <f>SUMIF(SalesTable[Region],D3,SalesTable[Total Sales])</f>
+        <v>9740</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>128</v>
       </c>
@@ -1305,8 +1328,15 @@
         <f>COUNTA(SalesTable[Order ID])</f>
         <v>50</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <f>SUMIF(SalesTable[Region],D4,SalesTable[Total Sales])</f>
+        <v>10705</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -1314,8 +1344,15 @@
         <f>AVEDEV(SalesTable[Total Sales])</f>
         <v>485.89600000000007</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <f>SUMIF(SalesTable[Region],D5,SalesTable[Total Sales])</f>
+        <v>12795</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>130</v>
       </c>
@@ -1324,7 +1361,7 @@
         <v>2550</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>131</v>
       </c>

</xml_diff>

<commit_message>
Use SUMIF for other calculations and Use SUMIFs function to calculate totals sales for each month
</commit_message>
<xml_diff>
--- a/Sales_Performance_Analysis.xlsx
+++ b/Sales_Performance_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI-Projects\sales-performance-analysis-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DD19108-D6E8-4AF6-A488-C6CFA3FF5340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD6C0A9-8532-4ED5-A28A-CCCF859B872F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="2" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="138">
   <si>
     <t>Region</t>
   </si>
@@ -437,6 +437,21 @@
   </si>
   <si>
     <t>Sales</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>January</t>
+  </si>
+  <si>
+    <t>February</t>
+  </si>
+  <si>
+    <t>March</t>
+  </si>
+  <si>
+    <t>April</t>
   </si>
 </sst>
 </file>
@@ -1267,14 +1282,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D65C6-FEF1-4656-8613-EFBCAEDD2EBF}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.77734375" customWidth="1"/>
     <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="14" max="14" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>125</v>
       </c>
@@ -1287,8 +1305,32 @@
       <c r="E1" s="11" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G1" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="P1" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="Q1" s="11" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -1303,8 +1345,36 @@
         <f>SUMIF(SalesTable[Region],D2,SalesTable[Total Sales])</f>
         <v>12045</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2">
+        <f>SUMIF(SalesTable[Salesperson],G2,SalesTable[Total Sales])</f>
+        <v>7595</v>
+      </c>
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2">
+        <f>SUMIF(SalesTable[Product],J2,SalesTable[Total Sales])</f>
+        <v>15300</v>
+      </c>
+      <c r="M2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N2">
+        <f>SUMIF(SalesTable[Category],M2,SalesTable[Total Sales])</f>
+        <v>22020</v>
+      </c>
+      <c r="P2" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q2">
+        <f>SUMIFS(SalesTable[Total Sales],SalesTable[Date],"&gt;="&amp;DATE(2026,1,1),SalesTable[Date],"&lt;"&amp;DATE(2026,2,1))</f>
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>127</v>
       </c>
@@ -1319,8 +1389,36 @@
         <f>SUMIF(SalesTable[Region],D3,SalesTable[Total Sales])</f>
         <v>9740</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3">
+        <f>SUMIF(SalesTable[Salesperson],G3,SalesTable[Total Sales])</f>
+        <v>5620</v>
+      </c>
+      <c r="J3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3">
+        <f>SUMIF(SalesTable[Product],J3,SalesTable[Total Sales])</f>
+        <v>6720</v>
+      </c>
+      <c r="M3" t="s">
+        <v>25</v>
+      </c>
+      <c r="N3">
+        <f>SUMIF(SalesTable[Category],M3,SalesTable[Total Sales])</f>
+        <v>6260</v>
+      </c>
+      <c r="P3" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q3">
+        <f>SUMIFS(SalesTable[Total Sales],SalesTable[Date],"&gt;="&amp;DATE(2026,2,1),SalesTable[Date],"&lt;"&amp;DATE(2026,3,1))</f>
+        <v>2635</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>128</v>
       </c>
@@ -1335,8 +1433,36 @@
         <f>SUMIF(SalesTable[Region],D4,SalesTable[Total Sales])</f>
         <v>10705</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4">
+        <f>SUMIF(SalesTable[Salesperson],G4,SalesTable[Total Sales])</f>
+        <v>4470</v>
+      </c>
+      <c r="J4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4">
+        <f>SUMIF(SalesTable[Product],J4,SalesTable[Total Sales])</f>
+        <v>1845</v>
+      </c>
+      <c r="M4" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4">
+        <f>SUMIF(SalesTable[Category],M4,SalesTable[Total Sales])</f>
+        <v>3075</v>
+      </c>
+      <c r="P4" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q4">
+        <f>SUMIFS(SalesTable[Total Sales],SalesTable[Date],"&gt;="&amp;DATE(2026,3,1),SalesTable[Date],"&lt;"&amp;DATE(2026,4,1))</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>129</v>
       </c>
@@ -1351,8 +1477,36 @@
         <f>SUMIF(SalesTable[Region],D5,SalesTable[Total Sales])</f>
         <v>12795</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5">
+        <f>SUMIF(SalesTable[Salesperson],G5,SalesTable[Total Sales])</f>
+        <v>5130</v>
+      </c>
+      <c r="J5" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5">
+        <f>SUMIF(SalesTable[Product],J5,SalesTable[Total Sales])</f>
+        <v>2075</v>
+      </c>
+      <c r="M5" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5">
+        <f>SUMIF(SalesTable[Category],M5,SalesTable[Total Sales])</f>
+        <v>4480</v>
+      </c>
+      <c r="P5" t="s">
+        <v>137</v>
+      </c>
+      <c r="Q5">
+        <f>SUMIFS(SalesTable[Total Sales],SalesTable[Date],"&gt;="&amp;DATE(2026,4,1),SalesTable[Date],"&lt;"&amp;DATE(2026,5,1))</f>
+        <v>2920</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>130</v>
       </c>
@@ -1360,14 +1514,81 @@
         <f>MAX(SalesTable[Total Sales])</f>
         <v>2550</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6">
+        <f>SUMIF(SalesTable[Salesperson],G6,SalesTable[Total Sales])</f>
+        <v>4450</v>
+      </c>
+      <c r="J6" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6">
+        <f>SUMIF(SalesTable[Product],J6,SalesTable[Total Sales])</f>
+        <v>3075</v>
+      </c>
+      <c r="M6" t="s">
+        <v>28</v>
+      </c>
+      <c r="N6">
+        <f>SUMIF(SalesTable[Category],M6,SalesTable[Total Sales])</f>
+        <v>9450</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>131</v>
       </c>
       <c r="B7">
         <f>MIN(SalesTable[Total Sales])</f>
         <v>200</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7">
+        <f>SUMIF(SalesTable[Salesperson],G7,SalesTable[Total Sales])</f>
+        <v>4120</v>
+      </c>
+      <c r="J7" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7">
+        <f>SUMIF(SalesTable[Product],J7,SalesTable[Total Sales])</f>
+        <v>4480</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8">
+        <f>SUMIF(SalesTable[Salesperson],G8,SalesTable[Total Sales])</f>
+        <v>6235</v>
+      </c>
+      <c r="J8" t="s">
+        <v>21</v>
+      </c>
+      <c r="K8">
+        <f>SUMIF(SalesTable[Product],J8,SalesTable[Total Sales])</f>
+        <v>2340</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9">
+        <f>SUMIF(SalesTable[Salesperson],G9,SalesTable[Total Sales])</f>
+        <v>7665</v>
+      </c>
+      <c r="J9" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9">
+        <f>SUMIF(SalesTable[Product],J9,SalesTable[Total Sales])</f>
+        <v>9450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Create sales analysis sheet with five Summary Tables
</commit_message>
<xml_diff>
--- a/Sales_Performance_Analysis.xlsx
+++ b/Sales_Performance_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI-Projects\sales-performance-analysis-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD6C0A9-8532-4ED5-A28A-CCCF859B872F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42C9FCE-C870-4A6E-A763-65D47B26F5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="2" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="145">
   <si>
     <t>Region</t>
   </si>
@@ -452,6 +452,27 @@
   </si>
   <si>
     <t>April</t>
+  </si>
+  <si>
+    <t>Sales Performance Analysis</t>
+  </si>
+  <si>
+    <t>Sales by Region</t>
+  </si>
+  <si>
+    <t>Sales by Product</t>
+  </si>
+  <si>
+    <t>Total  Sales</t>
+  </si>
+  <si>
+    <t>Sales by Category</t>
+  </si>
+  <si>
+    <t>Salesperson Performance</t>
+  </si>
+  <si>
+    <t>Monthly Sales</t>
   </si>
 </sst>
 </file>
@@ -461,7 +482,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$LKR]\ #,##0.00;[Red][$LKR]\ #,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -480,6 +501,14 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -527,7 +556,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -546,6 +575,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1273,9 +1303,307 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DE9B18C-9F45-4B2D-B24C-4271EB14C90A}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="12.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="A1" s="14" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G4" t="s">
+        <v>133</v>
+      </c>
+      <c r="H4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <f>Calculations!E2</f>
+        <v>12045</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5">
+        <f>Calculations!N2</f>
+        <v>22020</v>
+      </c>
+      <c r="G5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H5">
+        <f>Calculations!Q2</f>
+        <v>3300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6">
+        <f>Calculations!E3</f>
+        <v>9740</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <f>Calculations!N3</f>
+        <v>6260</v>
+      </c>
+      <c r="G6" t="s">
+        <v>135</v>
+      </c>
+      <c r="H6">
+        <f>Calculations!Q3</f>
+        <v>2635</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <f>Calculations!E4</f>
+        <v>10705</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7">
+        <f>Calculations!N4</f>
+        <v>3075</v>
+      </c>
+      <c r="G7" t="s">
+        <v>136</v>
+      </c>
+      <c r="H7">
+        <f>Calculations!Q4</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8">
+        <f>Calculations!E5</f>
+        <v>12795</v>
+      </c>
+      <c r="D8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8">
+        <f>Calculations!N5</f>
+        <v>4480</v>
+      </c>
+      <c r="G8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8">
+        <f>Calculations!Q5</f>
+        <v>2920</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9">
+        <f>Calculations!N6</f>
+        <v>9450</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12">
+        <f>Calculations!K2</f>
+        <v>15300</v>
+      </c>
+      <c r="D12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13">
+        <f>Calculations!K3</f>
+        <v>6720</v>
+      </c>
+      <c r="D13" t="s">
+        <v>6</v>
+      </c>
+      <c r="E13">
+        <f>Calculations!H2</f>
+        <v>7595</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14">
+        <f>Calculations!K4</f>
+        <v>1845</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14">
+        <f>Calculations!H3</f>
+        <v>5620</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15">
+        <f>Calculations!K5</f>
+        <v>2075</v>
+      </c>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15">
+        <f>Calculations!H4</f>
+        <v>4470</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16">
+        <f>Calculations!K6</f>
+        <v>3075</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <f>Calculations!H5</f>
+        <v>5130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17">
+        <f>Calculations!K7</f>
+        <v>4480</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17">
+        <f>Calculations!H6</f>
+        <v>4450</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18">
+        <f>Calculations!K8</f>
+        <v>2340</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18">
+        <f>Calculations!H7</f>
+        <v>4120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19">
+        <f>Calculations!K9</f>
+        <v>9450</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19">
+        <f>Calculations!H8</f>
+        <v>6235</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20">
+        <f>Calculations!H9</f>
+        <v>7665</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add different charts for Data Analysis perpose
</commit_message>
<xml_diff>
--- a/Sales_Performance_Analysis.xlsx
+++ b/Sales_Performance_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI-Projects\sales-performance-analysis-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A42C9FCE-C870-4A6E-A763-65D47B26F5FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C9B659-8991-4BAC-99B1-B2431D537DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
   </bookViews>
@@ -975,6 +975,4572 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Sales by Region</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$B$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$A$5:$A$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>North</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>South</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>East</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>West</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$B$5:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>12045</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9740</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10705</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12795</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2D48-4934-BF01-C5EB0208FB67}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="2018497520"/>
+        <c:axId val="2021543760"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="2018497520"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2021543760"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2021543760"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2018497520"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Sales by Product</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$B$11</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total  Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$A$12:$A$19</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Laptop</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Monitor</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Keyboard</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Mouse</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Headphones</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Printer</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Webcam</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Tablet</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$B$12:$B$19</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>15300</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6720</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1845</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2075</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>3075</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4480</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2340</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>9450</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E7C0-4589-B047-469FE5233A31}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="50174496"/>
+        <c:axId val="2021563920"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50174496"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2021563920"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="2021563920"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50174496"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Monthly Sales Trend</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$H$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$G$5:$G$8</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>January</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>February</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>March</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>April</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$H$5:$H$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3300</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2635</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>225</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2920</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3BD0-4778-936E-31DF62EBB800}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:smooth val="0"/>
+        <c:axId val="2019551200"/>
+        <c:axId val="42252176"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="2019551200"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="42252176"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="42252176"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="2019551200"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Sales by Category</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:doughnutChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$E$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$D$5:$D$9</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Computers</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Accessories</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Audio</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Office</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Mobile</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$E$5:$E$9</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>22020</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6260</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3075</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4480</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9450</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-C974-4F1E-84C7-8D910FE791EF}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+        <c:holeSize val="75"/>
+      </c:doughnutChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Salesperson Performance</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Analysis!$E$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total Sales</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Analysis!$D$13:$D$20</c:f>
+              <c:strCache>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>Dilusha</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sarath</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Minol</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Enul</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Dasun</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Senuri</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Devid</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Oshada</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Analysis!$E$13:$E$20</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="8"/>
+                <c:pt idx="0">
+                  <c:v>7595</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5620</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4470</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>5130</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4450</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4120</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6235</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7665</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6D7C-4825-97BB-BB002FF2DF56}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="35152432"/>
+        <c:axId val="42236336"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="35152432"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="42236336"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="42236336"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="35152432"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>1503</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>2919</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>316464</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>2920</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{725F24B5-F3A9-72DF-37F6-92C7AE0B4E3D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>-1</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>174811</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>283882</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>49306</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9C936C0-8A22-A883-2019-7D47133A89C3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>14940</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>174810</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>298823</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>49305</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{357A3666-066E-7572-4127-8F423BD41BE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>612587</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>8610</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>329045</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>92430</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E31182A-1098-F984-B7EC-17D67F9617A6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>770</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>4167</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>286836</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>171844</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Chart 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39D1519A-B75F-8C31-2FDD-5573375168CE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{56EF8F25-73E6-4863-9BA8-DBE529445E76}" name="SalesTable" displayName="SalesTable" ref="A1:K51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" tableBorderDxfId="12">
   <autoFilter ref="A1:K51" xr:uid="{56EF8F25-73E6-4863-9BA8-DBE529445E76}"/>
@@ -1605,6 +6171,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Create KPI card structure (5 Cards)
</commit_message>
<xml_diff>
--- a/Sales_Performance_Analysis.xlsx
+++ b/Sales_Performance_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI-Projects\sales-performance-analysis-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61C9B659-8991-4BAC-99B1-B2431D537DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A858F0-5451-4D69-A3C5-CB563AB47526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="153">
   <si>
     <t>Region</t>
   </si>
@@ -473,16 +473,41 @@
   </si>
   <si>
     <t>Monthly Sales</t>
+  </si>
+  <si>
+    <t>NOVA TECH SOLUTIONS</t>
+  </si>
+  <si>
+    <t>January - April 2026</t>
+  </si>
+  <si>
+    <t>SALES PERFORMANCE DASHBOARD</t>
+  </si>
+  <si>
+    <t>TOTAL SALES</t>
+  </si>
+  <si>
+    <t>TOTAL ORDERS</t>
+  </si>
+  <si>
+    <t>UNITS SOLD</t>
+  </si>
+  <si>
+    <t>AVG ORDER VALUE</t>
+  </si>
+  <si>
+    <t>HIGHEST SALE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$LKR]\ #,##0.00;[Red][$LKR]\ #,##0.00"/>
+    <numFmt numFmtId="168" formatCode="[$LKR]\ #,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -509,6 +534,36 @@
     <font>
       <b/>
       <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -556,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -576,6 +631,29 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2058,6 +2136,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-F013-40A8-AF93-3F8980E028CE}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -2073,6 +2156,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-F013-40A8-AF93-3F8980E028CE}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -2088,6 +2176,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-F013-40A8-AF93-3F8980E028CE}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -2103,6 +2196,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-F013-40A8-AF93-3F8980E028CE}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -2118,6 +2216,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-F013-40A8-AF93-3F8980E028CE}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:cat>
             <c:strRef>
@@ -5860,9 +5963,121 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30E678CE-0F2F-4A54-9D61-992795E3777A}">
-  <dimension ref="A1"/>
+  <dimension ref="B2:O8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="2:15" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="B2" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+    </row>
+    <row r="3" spans="2:15" ht="21" x14ac:dyDescent="0.4">
+      <c r="B3" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+    </row>
+    <row r="4" spans="2:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+    </row>
+    <row r="6" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B6" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="F6" s="18"/>
+      <c r="H6" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="I6" s="18"/>
+      <c r="K6" s="23" t="s">
+        <v>151</v>
+      </c>
+      <c r="L6" s="23"/>
+      <c r="N6" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="O6" s="18"/>
+    </row>
+    <row r="7" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B7" s="19">
+        <f>Calculations!B2</f>
+        <v>45285</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="18">
+        <f>Calculations!B4</f>
+        <v>50</v>
+      </c>
+      <c r="F7" s="18"/>
+      <c r="H7" s="22">
+        <f>Calculations!B3</f>
+        <v>277</v>
+      </c>
+      <c r="I7" s="18"/>
+      <c r="K7" s="18">
+        <f>Calculations!B5</f>
+        <v>485.89600000000007</v>
+      </c>
+      <c r="L7" s="18"/>
+      <c r="N7" s="18">
+        <f>Calculations!B6</f>
+        <v>2550</v>
+      </c>
+      <c r="O7" s="18"/>
+    </row>
+    <row r="8" spans="2:15" x14ac:dyDescent="0.3">
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="N8" s="18"/>
+      <c r="O8" s="18"/>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="N7:O8"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="E7:F8"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H7:I8"/>
+    <mergeCell ref="K6:L6"/>
+    <mergeCell ref="K7:L8"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="B7:C8"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -6184,6 +6399,7 @@
     <col min="2" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" customWidth="1"/>
     <col min="14" max="14" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
feat: add 5 core analytical charts to sales dashboard - Add line chart for monthly sales trend from summaty calculations - Add column chart for sales by region with data labes enabled - Add bar chart for sales by product sorted for horizontal readability - Add doughnut chart for sales by category distribution - Add column chart for salesperson performance tracking - Reorganize dashboard layout and sort source calculation tables from high to low
</commit_message>
<xml_diff>
--- a/Sales_Performance_Analysis.xlsx
+++ b/Sales_Performance_Analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BI-Projects\sales-performance-analysis-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46DE372-2A3C-4D86-B5DB-D24F9BB8F460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9C8D39-68D7-42AF-BBC5-A47F17F5C0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B7497976-6BF0-42CC-AA8A-1BF9F284EB1D}"/>
   </bookViews>
@@ -1867,6 +1867,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Calculations!$D$2:$D$5</c:f>
@@ -1915,8 +1973,9 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>

</xml_diff>